<commit_message>
🤖 자동 수집: 2026-09-06 09:47 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5913,6 +5913,28 @@
       </c>
       <c r="F62" t="n">
         <v>15.6</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-09-06T09:47:26.357181+09:00</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>0</v>
+      </c>
+      <c r="C63" t="n">
+        <v>0</v>
+      </c>
+      <c r="D63" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" t="n">
+        <v>15.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-07 09:50 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5935,6 +5935,28 @@
       </c>
       <c r="F63" t="n">
         <v>15.2</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:50:35.673568+09:00</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>0</v>
+      </c>
+      <c r="C64" t="n">
+        <v>0</v>
+      </c>
+      <c r="D64" t="n">
+        <v>0</v>
+      </c>
+      <c r="E64" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" t="n">
+        <v>14.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-08 10:06 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5957,6 +5957,28 @@
       </c>
       <c r="F64" t="n">
         <v>14.9</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-09-08T10:05:44.490819+09:00</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>0</v>
+      </c>
+      <c r="C65" t="n">
+        <v>0</v>
+      </c>
+      <c r="D65" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" t="n">
+        <v>16.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-09 10:09 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5979,6 +5979,28 @@
       </c>
       <c r="F65" t="n">
         <v>16.1</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-09-09T10:09:14.897990+09:00</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>0</v>
+      </c>
+      <c r="C66" t="n">
+        <v>0</v>
+      </c>
+      <c r="D66" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" t="n">
+        <v>18.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-10 09:58 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6001,6 +6001,28 @@
       </c>
       <c r="F66" t="n">
         <v>18.7</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-09-10T09:57:50.243638+09:00</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>0</v>
+      </c>
+      <c r="C67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" t="n">
+        <v>14.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-11 09:54 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F67"/>
+  <dimension ref="A1:F68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6023,6 +6023,28 @@
       </c>
       <c r="F67" t="n">
         <v>14.7</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-09-11T09:54:34.999385+09:00</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>0</v>
+      </c>
+      <c r="C68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" t="n">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-13 09:47 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6045,6 +6045,28 @@
       </c>
       <c r="F68" t="n">
         <v>16</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-09-13T09:47:07.634184+09:00</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>0</v>
+      </c>
+      <c r="C69" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" t="n">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-14 09:54 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6067,6 +6067,28 @@
       </c>
       <c r="F69" t="n">
         <v>15</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-09-14T09:53:45.113076+09:00</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>0</v>
+      </c>
+      <c r="C70" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" t="n">
+        <v>16.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-15 10:21 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F70"/>
+  <dimension ref="A1:F71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6089,6 +6089,28 @@
       </c>
       <c r="F70" t="n">
         <v>16.3</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-09-15T10:20:47.726473+09:00</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>0</v>
+      </c>
+      <c r="C71" t="n">
+        <v>0</v>
+      </c>
+      <c r="D71" t="n">
+        <v>0</v>
+      </c>
+      <c r="E71" t="n">
+        <v>0</v>
+      </c>
+      <c r="F71" t="n">
+        <v>15.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-16 10:16 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6111,6 +6111,28 @@
       </c>
       <c r="F71" t="n">
         <v>15.4</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-09-16T10:16:01.284629+09:00</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>0</v>
+      </c>
+      <c r="C72" t="n">
+        <v>0</v>
+      </c>
+      <c r="D72" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" t="n">
+        <v>0</v>
+      </c>
+      <c r="F72" t="n">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-17 10:16 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F72"/>
+  <dimension ref="A1:F73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6132,6 +6132,28 @@
         <v>0</v>
       </c>
       <c r="F72" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-09-17T10:15:50.809950+09:00</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>0</v>
+      </c>
+      <c r="C73" t="n">
+        <v>0</v>
+      </c>
+      <c r="D73" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" t="n">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-18 10:11 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6155,6 +6155,28 @@
       </c>
       <c r="F73" t="n">
         <v>16</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-09-18T10:11:27.638876+09:00</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>0</v>
+      </c>
+      <c r="C74" t="n">
+        <v>0</v>
+      </c>
+      <c r="D74" t="n">
+        <v>0</v>
+      </c>
+      <c r="E74" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" t="n">
+        <v>14.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-19 10:06 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F74"/>
+  <dimension ref="A1:F75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6177,6 +6177,28 @@
       </c>
       <c r="F74" t="n">
         <v>14.9</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-09-19T10:05:59.054699+09:00</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>0</v>
+      </c>
+      <c r="C75" t="n">
+        <v>0</v>
+      </c>
+      <c r="D75" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" t="n">
+        <v>25.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-20 09:56 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F75"/>
+  <dimension ref="A1:F76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6199,6 +6199,28 @@
       </c>
       <c r="F75" t="n">
         <v>25.9</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-09-20T09:56:15.927278+09:00</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>0</v>
+      </c>
+      <c r="C76" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" t="n">
+        <v>0</v>
+      </c>
+      <c r="E76" t="n">
+        <v>0</v>
+      </c>
+      <c r="F76" t="n">
+        <v>25.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-21 09:58 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:F77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6221,6 +6221,28 @@
       </c>
       <c r="F76" t="n">
         <v>25.6</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-09-21T09:58:24.536719+09:00</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>0</v>
+      </c>
+      <c r="C77" t="n">
+        <v>0</v>
+      </c>
+      <c r="D77" t="n">
+        <v>0</v>
+      </c>
+      <c r="E77" t="n">
+        <v>0</v>
+      </c>
+      <c r="F77" t="n">
+        <v>16.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-22 10:33 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F77"/>
+  <dimension ref="A1:F78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6243,6 +6243,28 @@
       </c>
       <c r="F77" t="n">
         <v>16.8</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-09-22T10:33:19.130992+09:00</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>0</v>
+      </c>
+      <c r="C78" t="n">
+        <v>0</v>
+      </c>
+      <c r="D78" t="n">
+        <v>0</v>
+      </c>
+      <c r="E78" t="n">
+        <v>0</v>
+      </c>
+      <c r="F78" t="n">
+        <v>16.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-23 10:23 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F78"/>
+  <dimension ref="A1:F79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6265,6 +6265,28 @@
       </c>
       <c r="F78" t="n">
         <v>16.2</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-09-23T10:23:40.692579+09:00</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C79" t="n">
+        <v>0</v>
+      </c>
+      <c r="D79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E79" t="n">
+        <v>0</v>
+      </c>
+      <c r="F79" t="n">
+        <v>15.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-26 10:24 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F79"/>
+  <dimension ref="A1:F80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6287,6 +6287,28 @@
       </c>
       <c r="F79" t="n">
         <v>15.4</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-09-26T10:24:05.361898+09:00</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>0</v>
+      </c>
+      <c r="C80" t="n">
+        <v>0</v>
+      </c>
+      <c r="D80" t="n">
+        <v>0</v>
+      </c>
+      <c r="E80" t="n">
+        <v>0</v>
+      </c>
+      <c r="F80" t="n">
+        <v>16.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-27 10:17 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F80"/>
+  <dimension ref="A1:F81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6309,6 +6309,28 @@
       </c>
       <c r="F80" t="n">
         <v>16.2</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-09-27T10:17:19.436314+09:00</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>0</v>
+      </c>
+      <c r="C81" t="n">
+        <v>0</v>
+      </c>
+      <c r="D81" t="n">
+        <v>0</v>
+      </c>
+      <c r="E81" t="n">
+        <v>0</v>
+      </c>
+      <c r="F81" t="n">
+        <v>15.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-28 10:31 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F81"/>
+  <dimension ref="A1:F82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6331,6 +6331,28 @@
       </c>
       <c r="F81" t="n">
         <v>15.8</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-09-28T10:31:03.255045+09:00</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>0</v>
+      </c>
+      <c r="C82" t="n">
+        <v>0</v>
+      </c>
+      <c r="D82" t="n">
+        <v>0</v>
+      </c>
+      <c r="E82" t="n">
+        <v>0</v>
+      </c>
+      <c r="F82" t="n">
+        <v>16.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-29 11:33 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F82"/>
+  <dimension ref="A1:F83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6353,6 +6353,28 @@
       </c>
       <c r="F82" t="n">
         <v>16.4</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-09-29T11:33:05.048636+09:00</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>0</v>
+      </c>
+      <c r="C83" t="n">
+        <v>0</v>
+      </c>
+      <c r="D83" t="n">
+        <v>0</v>
+      </c>
+      <c r="E83" t="n">
+        <v>0</v>
+      </c>
+      <c r="F83" t="n">
+        <v>15.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-01 10:58 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F83"/>
+  <dimension ref="A1:F84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6375,6 +6375,28 @@
       </c>
       <c r="F83" t="n">
         <v>15.9</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-10-01T10:58:31.874144+09:00</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>0</v>
+      </c>
+      <c r="C84" t="n">
+        <v>0</v>
+      </c>
+      <c r="D84" t="n">
+        <v>0</v>
+      </c>
+      <c r="E84" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" t="n">
+        <v>15.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-02 11:06 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F84"/>
+  <dimension ref="A1:F85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6397,6 +6397,28 @@
       </c>
       <c r="F84" t="n">
         <v>15.5</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-10-02T11:06:33.336711+09:00</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>0</v>
+      </c>
+      <c r="C85" t="n">
+        <v>0</v>
+      </c>
+      <c r="D85" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" t="n">
+        <v>0</v>
+      </c>
+      <c r="F85" t="n">
+        <v>16.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-03 10:52 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F85"/>
+  <dimension ref="A1:F86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6419,6 +6419,28 @@
       </c>
       <c r="F85" t="n">
         <v>16.1</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-10-03T10:51:59.827665+09:00</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>0</v>
+      </c>
+      <c r="C86" t="n">
+        <v>0</v>
+      </c>
+      <c r="D86" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" t="n">
+        <v>14.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-04 11:30 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F86"/>
+  <dimension ref="A1:F87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6441,6 +6441,28 @@
       </c>
       <c r="F86" t="n">
         <v>14.3</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-10-04T11:30:34.921112+09:00</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>0</v>
+      </c>
+      <c r="C87" t="n">
+        <v>0</v>
+      </c>
+      <c r="D87" t="n">
+        <v>0</v>
+      </c>
+      <c r="E87" t="n">
+        <v>0</v>
+      </c>
+      <c r="F87" t="n">
+        <v>15.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-06 11:52 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F87"/>
+  <dimension ref="A1:F88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6463,6 +6463,28 @@
       </c>
       <c r="F87" t="n">
         <v>15.8</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-10-06T11:52:02.847208+09:00</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>0</v>
+      </c>
+      <c r="C88" t="n">
+        <v>0</v>
+      </c>
+      <c r="D88" t="n">
+        <v>0</v>
+      </c>
+      <c r="E88" t="n">
+        <v>0</v>
+      </c>
+      <c r="F88" t="n">
+        <v>14.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-07 11:13 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F88"/>
+  <dimension ref="A1:F89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6485,6 +6485,28 @@
       </c>
       <c r="F88" t="n">
         <v>14.4</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-10-07T11:12:48.105716+09:00</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>0</v>
+      </c>
+      <c r="C89" t="n">
+        <v>0</v>
+      </c>
+      <c r="D89" t="n">
+        <v>0</v>
+      </c>
+      <c r="E89" t="n">
+        <v>0</v>
+      </c>
+      <c r="F89" t="n">
+        <v>15.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-08 11:38 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F89"/>
+  <dimension ref="A1:F90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6507,6 +6507,28 @@
       </c>
       <c r="F89" t="n">
         <v>15.9</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-10-08T11:38:14.192105+09:00</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>0</v>
+      </c>
+      <c r="C90" t="n">
+        <v>0</v>
+      </c>
+      <c r="D90" t="n">
+        <v>0</v>
+      </c>
+      <c r="E90" t="n">
+        <v>0</v>
+      </c>
+      <c r="F90" t="n">
+        <v>15.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-09 11:54 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F90"/>
+  <dimension ref="A1:F91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6529,6 +6529,28 @@
       </c>
       <c r="F90" t="n">
         <v>15.2</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-10-09T11:53:55.536497+09:00</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>0</v>
+      </c>
+      <c r="C91" t="n">
+        <v>0</v>
+      </c>
+      <c r="D91" t="n">
+        <v>0</v>
+      </c>
+      <c r="E91" t="n">
+        <v>0</v>
+      </c>
+      <c r="F91" t="n">
+        <v>15.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-10 11:14 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F91"/>
+  <dimension ref="A1:F92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6551,6 +6551,28 @@
       </c>
       <c r="F91" t="n">
         <v>15.1</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-10-10T11:14:35.221053+09:00</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>0</v>
+      </c>
+      <c r="C92" t="n">
+        <v>0</v>
+      </c>
+      <c r="D92" t="n">
+        <v>0</v>
+      </c>
+      <c r="E92" t="n">
+        <v>0</v>
+      </c>
+      <c r="F92" t="n">
+        <v>18.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-11 10:46 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F92"/>
+  <dimension ref="A1:F93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6573,6 +6573,28 @@
       </c>
       <c r="F92" t="n">
         <v>18.1</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-10-11T10:46:37.262669+09:00</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>0</v>
+      </c>
+      <c r="C93" t="n">
+        <v>0</v>
+      </c>
+      <c r="D93" t="n">
+        <v>0</v>
+      </c>
+      <c r="E93" t="n">
+        <v>0</v>
+      </c>
+      <c r="F93" t="n">
+        <v>14.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-12 11:14 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F93"/>
+  <dimension ref="A1:F94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6595,6 +6595,28 @@
       </c>
       <c r="F93" t="n">
         <v>14.7</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-10-12T11:14:05.850748+09:00</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>0</v>
+      </c>
+      <c r="C94" t="n">
+        <v>0</v>
+      </c>
+      <c r="D94" t="n">
+        <v>0</v>
+      </c>
+      <c r="E94" t="n">
+        <v>0</v>
+      </c>
+      <c r="F94" t="n">
+        <v>14.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-13 12:28 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F94"/>
+  <dimension ref="A1:F95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6617,6 +6617,28 @@
       </c>
       <c r="F94" t="n">
         <v>14.1</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-10-13T12:28:16.318593+09:00</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>0</v>
+      </c>
+      <c r="C95" t="n">
+        <v>0</v>
+      </c>
+      <c r="D95" t="n">
+        <v>0</v>
+      </c>
+      <c r="E95" t="n">
+        <v>0</v>
+      </c>
+      <c r="F95" t="n">
+        <v>16.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-14 10:46 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F95"/>
+  <dimension ref="A1:F96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6639,6 +6639,28 @@
       </c>
       <c r="F95" t="n">
         <v>16.8</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-10-14T10:46:27.618960+09:00</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>0</v>
+      </c>
+      <c r="C96" t="n">
+        <v>0</v>
+      </c>
+      <c r="D96" t="n">
+        <v>0</v>
+      </c>
+      <c r="E96" t="n">
+        <v>0</v>
+      </c>
+      <c r="F96" t="n">
+        <v>14.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-15 10:22 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F96"/>
+  <dimension ref="A1:F97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6661,6 +6661,28 @@
       </c>
       <c r="F96" t="n">
         <v>14.5</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-10-15T10:21:57.853136+09:00</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>0</v>
+      </c>
+      <c r="C97" t="n">
+        <v>0</v>
+      </c>
+      <c r="D97" t="n">
+        <v>0</v>
+      </c>
+      <c r="E97" t="n">
+        <v>0</v>
+      </c>
+      <c r="F97" t="n">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-16 10:08 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F97"/>
+  <dimension ref="A1:F98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6683,6 +6683,28 @@
       </c>
       <c r="F97" t="n">
         <v>15</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-10-16T10:08:29.032914+09:00</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>0</v>
+      </c>
+      <c r="C98" t="n">
+        <v>0</v>
+      </c>
+      <c r="D98" t="n">
+        <v>0</v>
+      </c>
+      <c r="E98" t="n">
+        <v>0</v>
+      </c>
+      <c r="F98" t="n">
+        <v>16.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-18 09:49 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F98"/>
+  <dimension ref="A1:F99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6705,6 +6705,28 @@
       </c>
       <c r="F98" t="n">
         <v>16.4</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-10-18T09:49:01.398682+09:00</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>0</v>
+      </c>
+      <c r="C99" t="n">
+        <v>0</v>
+      </c>
+      <c r="D99" t="n">
+        <v>0</v>
+      </c>
+      <c r="E99" t="n">
+        <v>0</v>
+      </c>
+      <c r="F99" t="n">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-19 10:04 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F99"/>
+  <dimension ref="A1:F100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6727,6 +6727,28 @@
       </c>
       <c r="F99" t="n">
         <v>17</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-10-19T10:03:57.565967+09:00</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>0</v>
+      </c>
+      <c r="C100" t="n">
+        <v>0</v>
+      </c>
+      <c r="D100" t="n">
+        <v>0</v>
+      </c>
+      <c r="E100" t="n">
+        <v>0</v>
+      </c>
+      <c r="F100" t="n">
+        <v>16.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-20 10:41 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F100"/>
+  <dimension ref="A1:F101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6749,6 +6749,28 @@
       </c>
       <c r="F100" t="n">
         <v>16.7</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-10-20T10:41:01.296281+09:00</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>0</v>
+      </c>
+      <c r="C101" t="n">
+        <v>0</v>
+      </c>
+      <c r="D101" t="n">
+        <v>0</v>
+      </c>
+      <c r="E101" t="n">
+        <v>0</v>
+      </c>
+      <c r="F101" t="n">
+        <v>19.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-21 10:26 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:F102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6771,6 +6771,28 @@
       </c>
       <c r="F101" t="n">
         <v>19.5</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-10-21T10:26:17.758085+09:00</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>0</v>
+      </c>
+      <c r="C102" t="n">
+        <v>0</v>
+      </c>
+      <c r="D102" t="n">
+        <v>0</v>
+      </c>
+      <c r="E102" t="n">
+        <v>0</v>
+      </c>
+      <c r="F102" t="n">
+        <v>17.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-22 10:25 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F102"/>
+  <dimension ref="A1:F103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6793,6 +6793,28 @@
       </c>
       <c r="F102" t="n">
         <v>17.6</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-10-22T10:24:45.051676+09:00</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>0</v>
+      </c>
+      <c r="C103" t="n">
+        <v>0</v>
+      </c>
+      <c r="D103" t="n">
+        <v>0</v>
+      </c>
+      <c r="E103" t="n">
+        <v>0</v>
+      </c>
+      <c r="F103" t="n">
+        <v>17.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-23 10:23 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F103"/>
+  <dimension ref="A1:F104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6815,6 +6815,28 @@
       </c>
       <c r="F103" t="n">
         <v>17.4</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-10-23T10:22:49.982841+09:00</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>0</v>
+      </c>
+      <c r="C104" t="n">
+        <v>0</v>
+      </c>
+      <c r="D104" t="n">
+        <v>0</v>
+      </c>
+      <c r="E104" t="n">
+        <v>0</v>
+      </c>
+      <c r="F104" t="n">
+        <v>20.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-24 10:29 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F104"/>
+  <dimension ref="A1:F105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6837,6 +6837,28 @@
       </c>
       <c r="F104" t="n">
         <v>20.3</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-10-24T10:28:39.530958+09:00</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>0</v>
+      </c>
+      <c r="C105" t="n">
+        <v>0</v>
+      </c>
+      <c r="D105" t="n">
+        <v>0</v>
+      </c>
+      <c r="E105" t="n">
+        <v>0</v>
+      </c>
+      <c r="F105" t="n">
+        <v>20.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-25 09:59 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F105"/>
+  <dimension ref="A1:F106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6859,6 +6859,28 @@
       </c>
       <c r="F105" t="n">
         <v>20.5</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-10-25T09:58:56.787144+09:00</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>0</v>
+      </c>
+      <c r="C106" t="n">
+        <v>0</v>
+      </c>
+      <c r="D106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F106" t="n">
+        <v>19.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-26 10:06 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F106"/>
+  <dimension ref="A1:F107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6881,6 +6881,28 @@
       </c>
       <c r="F106" t="n">
         <v>19.7</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-10-26T10:05:40.343272+09:00</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>0</v>
+      </c>
+      <c r="C107" t="n">
+        <v>0</v>
+      </c>
+      <c r="D107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E107" t="n">
+        <v>0</v>
+      </c>
+      <c r="F107" t="n">
+        <v>20.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-28 11:06 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F107"/>
+  <dimension ref="A1:F108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6903,6 +6903,28 @@
       </c>
       <c r="F107" t="n">
         <v>20.7</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-10-28T11:06:20.321518+09:00</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>0</v>
+      </c>
+      <c r="C108" t="n">
+        <v>0</v>
+      </c>
+      <c r="D108" t="n">
+        <v>0</v>
+      </c>
+      <c r="E108" t="n">
+        <v>0</v>
+      </c>
+      <c r="F108" t="n">
+        <v>18.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-29 11:18 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F108"/>
+  <dimension ref="A1:F109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6925,6 +6925,28 @@
       </c>
       <c r="F108" t="n">
         <v>18.5</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-10-29T11:18:00.575489+09:00</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>0</v>
+      </c>
+      <c r="C109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E109" t="n">
+        <v>0</v>
+      </c>
+      <c r="F109" t="n">
+        <v>17.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-30 11:30 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F109"/>
+  <dimension ref="A1:F110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6947,6 +6947,28 @@
       </c>
       <c r="F109" t="n">
         <v>17.2</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-10-30T11:30:03.564372+09:00</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>0</v>
+      </c>
+      <c r="C110" t="n">
+        <v>0</v>
+      </c>
+      <c r="D110" t="n">
+        <v>0</v>
+      </c>
+      <c r="E110" t="n">
+        <v>0</v>
+      </c>
+      <c r="F110" t="n">
+        <v>16.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-10-31 11:13 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F110"/>
+  <dimension ref="A1:F111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6969,6 +6969,28 @@
       </c>
       <c r="F110" t="n">
         <v>16.4</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-10-31T11:13:10.553560+09:00</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>0</v>
+      </c>
+      <c r="C111" t="n">
+        <v>0</v>
+      </c>
+      <c r="D111" t="n">
+        <v>0</v>
+      </c>
+      <c r="E111" t="n">
+        <v>0</v>
+      </c>
+      <c r="F111" t="n">
+        <v>18.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>